<commit_message>
Update aaa-quiver score statistics spreadsheet
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/aaa-quiver/分数统计.xlsx
+++ b/aaa-quiver/分数统计.xlsx
@@ -1,13 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2026spring\aaa-quiver\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF57A850-199C-4A36-B8A3-EEF0C7998259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="27570" windowHeight="15225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,9 +25,222 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="54">
+  <si>
+    <t>2026春季学期点名册</t>
+  </si>
+  <si>
+    <t>课程号：MA235</t>
+  </si>
+  <si>
+    <t>课程名称：应用抽象代数</t>
+  </si>
+  <si>
+    <t>开课学院：数学系</t>
+  </si>
+  <si>
+    <t>任课教师：Iryna Kashuba</t>
+  </si>
+  <si>
+    <t>学分：3</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="SimSun"/>
+        <charset val="134"/>
+      </rPr>
+      <t>上课时间</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="12"/>
+        <rFont val="Dialog.bolditalic"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="SimSun"/>
+        <charset val="134"/>
+      </rPr>
+      <t>1-15周,星期一第3-4节 一教225</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="12"/>
+        <rFont val="Dialog.bolditalic"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="SimSun"/>
+        <charset val="134"/>
+      </rPr>
+      <t>1-15单周,星期三第3-4节 一教225</t>
+    </r>
+  </si>
+  <si>
+    <t>教学班名称</t>
+  </si>
+  <si>
+    <t>应用抽象代数-01班-英文</t>
+  </si>
+  <si>
+    <t>序号</t>
+  </si>
+  <si>
+    <t>学号</t>
+  </si>
+  <si>
+    <t>本/研</t>
+  </si>
+  <si>
+    <t>姓名</t>
+  </si>
+  <si>
+    <t>专业</t>
+  </si>
+  <si>
+    <t>班级</t>
+  </si>
+  <si>
+    <t>成绩</t>
+  </si>
+  <si>
+    <t>书院</t>
+  </si>
+  <si>
+    <t>备注</t>
+  </si>
+  <si>
+    <t>12010612</t>
+  </si>
+  <si>
+    <t>本</t>
+  </si>
+  <si>
+    <t>梁顺泰</t>
+  </si>
+  <si>
+    <t>数学与应用数学</t>
+  </si>
+  <si>
+    <t>20级数学与应用数学</t>
+  </si>
+  <si>
+    <t>树礼书院</t>
+  </si>
+  <si>
+    <t>已生效</t>
+  </si>
+  <si>
+    <t>12310227</t>
+  </si>
+  <si>
+    <t>戴震远</t>
+  </si>
+  <si>
+    <t>23级数学与应用数学</t>
+  </si>
+  <si>
+    <t>致新书院</t>
+  </si>
+  <si>
+    <t>12310325</t>
+  </si>
+  <si>
+    <t>万宇轩</t>
+  </si>
+  <si>
+    <t>12310609</t>
+  </si>
+  <si>
+    <t>朱丹</t>
+  </si>
+  <si>
+    <t>12311312</t>
+  </si>
+  <si>
+    <t>王琛</t>
+  </si>
+  <si>
+    <t>致诚书院</t>
+  </si>
+  <si>
+    <t>12312009</t>
+  </si>
+  <si>
+    <t>张心远</t>
+  </si>
+  <si>
+    <t>树德书院</t>
+  </si>
+  <si>
+    <t>12313317</t>
+  </si>
+  <si>
+    <t>王禹斌</t>
+  </si>
+  <si>
+    <t>致仁书院</t>
+  </si>
+  <si>
+    <t>12413211</t>
+  </si>
+  <si>
+    <t>王思忧</t>
+  </si>
+  <si>
+    <t>24级数学与应用数学</t>
+  </si>
+  <si>
+    <t>作业1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>作业2</t>
+  </si>
+  <si>
+    <t>作业3</t>
+  </si>
+  <si>
+    <t>作业4</t>
+  </si>
+  <si>
+    <t>作业5</t>
+  </si>
+  <si>
+    <t>作业6</t>
+  </si>
+  <si>
+    <t>作业7</t>
+  </si>
+  <si>
+    <t>期中</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>期末</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,16 +248,46 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="SimSun"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="SimSun"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="12"/>
+      <name val="Dialog.bolditalic"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC0C0C0"/>
+        <bgColor rgb="FFC0C0C0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,15 +295,51 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -330,10 +616,602 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="4.75" style="2" customWidth="1"/>
+    <col min="2" max="2" width="9.75" style="2" customWidth="1"/>
+    <col min="3" max="3" width="5.375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="9.75" style="2" customWidth="1"/>
+    <col min="5" max="5" width="5.875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="11.25" style="2" customWidth="1"/>
+    <col min="7" max="8" width="7.75" style="2" customWidth="1"/>
+    <col min="9" max="9" width="5.125" style="2" customWidth="1"/>
+    <col min="10" max="11" width="9.75" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="10" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="20.45" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" ht="14.25" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+    </row>
+    <row r="3" spans="1:11" ht="14.25" customHeight="1">
+      <c r="A3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" ht="57.95" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" ht="14.25" customHeight="1">
+      <c r="A5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" ht="14.25" customHeight="1">
+      <c r="A6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" s="4"/>
+      <c r="I6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="14.25" customHeight="1">
+      <c r="A7" s="6">
+        <v>1</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="7"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="14.25" customHeight="1">
+      <c r="A8" s="6">
+        <v>2</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="7"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="14.25" customHeight="1">
+      <c r="A9" s="6">
+        <v>3</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="7"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="14.25" customHeight="1">
+      <c r="A10" s="6">
+        <v>4</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="7"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="14.25" customHeight="1">
+      <c r="A11" s="6">
+        <v>5</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="7"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="14.25" customHeight="1">
+      <c r="A12" s="6">
+        <v>6</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" s="7"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="14.25" customHeight="1">
+      <c r="A13" s="6">
+        <v>7</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" s="7"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="14.25" customHeight="1">
+      <c r="A14" s="6">
+        <v>8</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H14" s="7"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="27">
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="D5:K5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="H2:K2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="H3:K3"/>
+  </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97D1970F-41D6-4816-8D53-5FDF798DA708}">
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="E1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1" t="s">
+        <v>49</v>
+      </c>
+      <c r="J1" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1" t="s">
+        <v>51</v>
+      </c>
+      <c r="L1" t="s">
+        <v>52</v>
+      </c>
+      <c r="M1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="6">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="6">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3">
+        <v>20</v>
+      </c>
+      <c r="F3">
+        <v>20</v>
+      </c>
+      <c r="L3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="6">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="L4">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="6">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5">
+        <v>20</v>
+      </c>
+      <c r="F5">
+        <v>20</v>
+      </c>
+      <c r="L5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6">
+        <v>20</v>
+      </c>
+      <c r="F6">
+        <v>20</v>
+      </c>
+      <c r="L6">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="6">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7">
+        <v>20</v>
+      </c>
+      <c r="F7">
+        <v>20</v>
+      </c>
+      <c r="L7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="6">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8">
+        <v>20</v>
+      </c>
+      <c r="F8">
+        <v>20</v>
+      </c>
+      <c r="L8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="6">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="L9">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>